<commit_message>
Add PiN results (Excel) for Burkina_Faso___BFA
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Burkina_Faso___BFA/PiN_results_Burkina_Faso___BFA_1009_10AM.xlsx
+++ b/platform_PiN_output/Burkina_Faso___BFA/PiN_results_Burkina_Faso___BFA_1009_10AM.xlsx
@@ -1105,7 +1105,7 @@
       <c r="D5" s="14" t="n"/>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>d_origine_admin3</t>
+          <t>admin1</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -13518,7 +13518,7 @@
       <c r="D5" s="14" t="n"/>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>d_origine_admin3</t>
+          <t>admin1</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -27191,7 +27191,7 @@
       <c r="D5" s="14" t="n"/>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>d_origine_admin3</t>
+          <t>admin1</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -40203,7 +40203,7 @@
       </c>
       <c r="G7" s="35" t="inlineStr">
         <is>
-          <t>09/10/2025 10:35</t>
+          <t>09/10/2025 10:43</t>
         </is>
       </c>
     </row>

</xml_diff>